<commit_message>
#16 #15 #14 eSpark and Client BOM Completed.
</commit_message>
<xml_diff>
--- a/Design-Files/OFP_MCM_v1.5/BOM/Client-BOM-OFP_MCM_v1.5.xlsx
+++ b/Design-Files/OFP_MCM_v1.5/BOM/Client-BOM-OFP_MCM_v1.5.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="951" uniqueCount="561">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="959" uniqueCount="565">
   <si>
     <t>#</t>
   </si>
@@ -1702,13 +1702,25 @@
   </si>
   <si>
     <t>MyAntenna</t>
+  </si>
+  <si>
+    <t>FPC FFC Flexible Flat Cable Extension Board PCB Pitch 0.5 mm (40 Pin) Connector</t>
+  </si>
+  <si>
+    <t>CA-2660</t>
+  </si>
+  <si>
+    <t>RZCONNE</t>
+  </si>
+  <si>
+    <t>Aliexpress</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1776,6 +1788,21 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color indexed="12"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color indexed="12"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -1797,7 +1824,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -1888,11 +1915,27 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="8"/>
+      </left>
+      <right style="thin">
+        <color indexed="8"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="8"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1944,8 +1987,12 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -2231,8 +2278,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K135"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:K136"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="4" style="4" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18.7109375" style="4" bestFit="1" customWidth="1"/>
@@ -2246,7 +2293,7 @@
     <col min="11" max="11" width="13.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="15.75" thickBot="1">
       <c r="A1" s="1"/>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -2259,7 +2306,7 @@
       <c r="J1" s="18"/>
       <c r="K1" s="18"/>
     </row>
-    <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" ht="15.75" thickBot="1">
       <c r="A2" s="1"/>
       <c r="B2" s="5" t="s">
         <v>0</v>
@@ -2292,7 +2339,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" ht="15.75" thickBot="1">
       <c r="A3" s="1"/>
       <c r="B3" s="11">
         <f>ROW(B3) - ROW($B$2)</f>
@@ -2324,7 +2371,7 @@
       </c>
       <c r="K3" s="7"/>
     </row>
-    <row r="4" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" ht="15.75" thickBot="1">
       <c r="A4" s="1"/>
       <c r="B4" s="11">
         <f t="shared" ref="B4:B131" si="0">ROW(B4) - ROW($B$2)</f>
@@ -2356,7 +2403,7 @@
       </c>
       <c r="K4" s="9"/>
     </row>
-    <row r="5" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" ht="24.75" thickBot="1">
       <c r="A5" s="1"/>
       <c r="B5" s="11">
         <f>ROW(B5) - ROW($B$2)</f>
@@ -2388,7 +2435,7 @@
       </c>
       <c r="K5" s="7"/>
     </row>
-    <row r="6" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" ht="48.75" thickBot="1">
       <c r="A6" s="1"/>
       <c r="B6" s="11">
         <f t="shared" si="0"/>
@@ -2420,7 +2467,7 @@
       </c>
       <c r="K6" s="9"/>
     </row>
-    <row r="7" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" ht="15.75" thickBot="1">
       <c r="A7" s="1"/>
       <c r="B7" s="11">
         <f>ROW(B7) - ROW($B$2)</f>
@@ -2452,7 +2499,7 @@
       </c>
       <c r="K7" s="7"/>
     </row>
-    <row r="8" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" ht="24.75" thickBot="1">
       <c r="A8" s="1"/>
       <c r="B8" s="11">
         <f t="shared" si="0"/>
@@ -2484,7 +2531,7 @@
       </c>
       <c r="K8" s="9"/>
     </row>
-    <row r="9" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" ht="15.75" thickBot="1">
       <c r="A9" s="1"/>
       <c r="B9" s="11">
         <f>ROW(B9) - ROW($B$2)</f>
@@ -2516,7 +2563,7 @@
       </c>
       <c r="K9" s="7"/>
     </row>
-    <row r="10" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" ht="15.75" thickBot="1">
       <c r="A10" s="1"/>
       <c r="B10" s="11">
         <f t="shared" si="0"/>
@@ -2548,7 +2595,7 @@
       </c>
       <c r="K10" s="9"/>
     </row>
-    <row r="11" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" ht="15.75" thickBot="1">
       <c r="A11" s="1"/>
       <c r="B11" s="11">
         <f>ROW(B11) - ROW($B$2)</f>
@@ -2580,7 +2627,7 @@
       </c>
       <c r="K11" s="7"/>
     </row>
-    <row r="12" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" ht="24.75" thickBot="1">
       <c r="A12" s="1"/>
       <c r="B12" s="11">
         <f t="shared" si="0"/>
@@ -2612,7 +2659,7 @@
       </c>
       <c r="K12" s="9"/>
     </row>
-    <row r="13" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" ht="15.75" thickBot="1">
       <c r="A13" s="1"/>
       <c r="B13" s="11">
         <f>ROW(B13) - ROW($B$2)</f>
@@ -2644,7 +2691,7 @@
       </c>
       <c r="K13" s="7"/>
     </row>
-    <row r="14" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" ht="15.75" thickBot="1">
       <c r="A14" s="1"/>
       <c r="B14" s="11">
         <f t="shared" si="0"/>
@@ -2676,7 +2723,7 @@
       </c>
       <c r="K14" s="9"/>
     </row>
-    <row r="15" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" ht="15.75" thickBot="1">
       <c r="A15" s="1"/>
       <c r="B15" s="11">
         <f>ROW(B15) - ROW($B$2)</f>
@@ -2708,7 +2755,7 @@
       </c>
       <c r="K15" s="7"/>
     </row>
-    <row r="16" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" ht="15.75" thickBot="1">
       <c r="A16" s="1"/>
       <c r="B16" s="11">
         <f t="shared" si="0"/>
@@ -2740,7 +2787,7 @@
       </c>
       <c r="K16" s="9"/>
     </row>
-    <row r="17" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" ht="15.75" thickBot="1">
       <c r="A17" s="1"/>
       <c r="B17" s="11">
         <f>ROW(B17) - ROW($B$2)</f>
@@ -2772,7 +2819,7 @@
       </c>
       <c r="K17" s="7"/>
     </row>
-    <row r="18" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" ht="15.75" thickBot="1">
       <c r="A18" s="1"/>
       <c r="B18" s="11">
         <f t="shared" si="0"/>
@@ -2804,7 +2851,7 @@
       </c>
       <c r="K18" s="9"/>
     </row>
-    <row r="19" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" ht="15.75" thickBot="1">
       <c r="A19" s="1"/>
       <c r="B19" s="11">
         <f>ROW(B19) - ROW($B$2)</f>
@@ -2836,7 +2883,7 @@
       </c>
       <c r="K19" s="7"/>
     </row>
-    <row r="20" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" ht="15.75" thickBot="1">
       <c r="A20" s="1"/>
       <c r="B20" s="11">
         <f t="shared" si="0"/>
@@ -2868,7 +2915,7 @@
       </c>
       <c r="K20" s="9"/>
     </row>
-    <row r="21" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" ht="15.75" thickBot="1">
       <c r="A21" s="1"/>
       <c r="B21" s="11">
         <f>ROW(B21) - ROW($B$2)</f>
@@ -2900,7 +2947,7 @@
       </c>
       <c r="K21" s="7"/>
     </row>
-    <row r="22" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" ht="15.75" thickBot="1">
       <c r="A22" s="1"/>
       <c r="B22" s="11">
         <f t="shared" si="0"/>
@@ -2932,7 +2979,7 @@
       </c>
       <c r="K22" s="9"/>
     </row>
-    <row r="23" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" ht="15.75" thickBot="1">
       <c r="A23" s="1"/>
       <c r="B23" s="11">
         <f>ROW(B23) - ROW($B$2)</f>
@@ -2964,7 +3011,7 @@
       </c>
       <c r="K23" s="7"/>
     </row>
-    <row r="24" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" ht="15.75" thickBot="1">
       <c r="A24" s="1"/>
       <c r="B24" s="11">
         <f t="shared" si="0"/>
@@ -2996,7 +3043,7 @@
       </c>
       <c r="K24" s="9"/>
     </row>
-    <row r="25" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" ht="15.75" thickBot="1">
       <c r="A25" s="1"/>
       <c r="B25" s="11">
         <f>ROW(B25) - ROW($B$2)</f>
@@ -3028,7 +3075,7 @@
       </c>
       <c r="K25" s="7"/>
     </row>
-    <row r="26" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" ht="15.75" thickBot="1">
       <c r="A26" s="1"/>
       <c r="B26" s="11">
         <f t="shared" si="0"/>
@@ -3060,7 +3107,7 @@
       </c>
       <c r="K26" s="9"/>
     </row>
-    <row r="27" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" ht="15.75" thickBot="1">
       <c r="A27" s="1"/>
       <c r="B27" s="11">
         <f>ROW(B27) - ROW($B$2)</f>
@@ -3092,7 +3139,7 @@
       </c>
       <c r="K27" s="7"/>
     </row>
-    <row r="28" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" ht="15.75" thickBot="1">
       <c r="A28" s="1"/>
       <c r="B28" s="11">
         <f t="shared" si="0"/>
@@ -3124,7 +3171,7 @@
       </c>
       <c r="K28" s="9"/>
     </row>
-    <row r="29" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" ht="15.75" thickBot="1">
       <c r="A29" s="1"/>
       <c r="B29" s="11">
         <f>ROW(B29) - ROW($B$2)</f>
@@ -3156,7 +3203,7 @@
       </c>
       <c r="K29" s="7"/>
     </row>
-    <row r="30" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" ht="15.75" thickBot="1">
       <c r="A30" s="1"/>
       <c r="B30" s="11">
         <f t="shared" si="0"/>
@@ -3188,7 +3235,7 @@
       </c>
       <c r="K30" s="9"/>
     </row>
-    <row r="31" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" ht="15.75" thickBot="1">
       <c r="A31" s="1"/>
       <c r="B31" s="11">
         <f>ROW(B31) - ROW($B$2)</f>
@@ -3220,7 +3267,7 @@
       </c>
       <c r="K31" s="7"/>
     </row>
-    <row r="32" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" ht="15.75" thickBot="1">
       <c r="A32" s="1"/>
       <c r="B32" s="11">
         <f t="shared" si="0"/>
@@ -3254,7 +3301,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="33" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" ht="15.75" thickBot="1">
       <c r="A33" s="1"/>
       <c r="B33" s="11">
         <f>ROW(B33) - ROW($B$2)</f>
@@ -3288,7 +3335,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="34" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11" ht="36.75" thickBot="1">
       <c r="A34" s="1"/>
       <c r="B34" s="11">
         <f t="shared" si="0"/>
@@ -3320,7 +3367,7 @@
       </c>
       <c r="K34" s="9"/>
     </row>
-    <row r="35" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:11" ht="24.75" thickBot="1">
       <c r="A35" s="1"/>
       <c r="B35" s="11">
         <f>ROW(B35) - ROW($B$2)</f>
@@ -3352,7 +3399,7 @@
       </c>
       <c r="K35" s="7"/>
     </row>
-    <row r="36" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:11" ht="15.75" thickBot="1">
       <c r="A36" s="1"/>
       <c r="B36" s="11">
         <f t="shared" si="0"/>
@@ -3386,7 +3433,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="37" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:11" ht="15.75" thickBot="1">
       <c r="A37" s="1"/>
       <c r="B37" s="11">
         <f>ROW(B37) - ROW($B$2)</f>
@@ -3418,7 +3465,7 @@
       </c>
       <c r="K37" s="7"/>
     </row>
-    <row r="38" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:11" ht="36.75" thickBot="1">
       <c r="A38" s="1"/>
       <c r="B38" s="11">
         <f t="shared" si="0"/>
@@ -3450,7 +3497,7 @@
       </c>
       <c r="K38" s="9"/>
     </row>
-    <row r="39" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:11" ht="48.75" thickBot="1">
       <c r="A39" s="1"/>
       <c r="B39" s="11">
         <f>ROW(B39) - ROW($B$2)</f>
@@ -3482,7 +3529,7 @@
       </c>
       <c r="K39" s="7"/>
     </row>
-    <row r="40" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:11" ht="24.75" thickBot="1">
       <c r="A40" s="1"/>
       <c r="B40" s="11">
         <f t="shared" si="0"/>
@@ -3514,7 +3561,7 @@
       </c>
       <c r="K40" s="9"/>
     </row>
-    <row r="41" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:11" ht="15.75" thickBot="1">
       <c r="A41" s="1"/>
       <c r="B41" s="11">
         <f>ROW(B41) - ROW($B$2)</f>
@@ -3546,7 +3593,7 @@
       </c>
       <c r="K41" s="7"/>
     </row>
-    <row r="42" spans="1:11" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:11" ht="26.25" thickBot="1">
       <c r="A42" s="1"/>
       <c r="B42" s="11">
         <f t="shared" si="0"/>
@@ -3578,7 +3625,7 @@
       </c>
       <c r="K42" s="9"/>
     </row>
-    <row r="43" spans="1:11" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:11" ht="26.25" thickBot="1">
       <c r="A43" s="1"/>
       <c r="B43" s="11">
         <f t="shared" si="0"/>
@@ -3612,7 +3659,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="44" spans="1:11" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:11" ht="26.25" thickBot="1">
       <c r="A44" s="1"/>
       <c r="B44" s="11">
         <f t="shared" si="0"/>
@@ -3644,7 +3691,7 @@
       </c>
       <c r="K44" s="9"/>
     </row>
-    <row r="45" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:11" ht="15.75" thickBot="1">
       <c r="A45" s="1"/>
       <c r="B45" s="11">
         <f t="shared" si="0"/>
@@ -3676,7 +3723,7 @@
       </c>
       <c r="K45" s="9"/>
     </row>
-    <row r="46" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:11" ht="24.75" thickBot="1">
       <c r="A46" s="1"/>
       <c r="B46" s="11">
         <f>ROW(B46) - ROW($B$2)</f>
@@ -3708,7 +3755,7 @@
       </c>
       <c r="K46" s="7"/>
     </row>
-    <row r="47" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:11" ht="15.75" thickBot="1">
       <c r="A47" s="1"/>
       <c r="B47" s="11">
         <f t="shared" si="0"/>
@@ -3740,7 +3787,7 @@
       </c>
       <c r="K47" s="9"/>
     </row>
-    <row r="48" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:11" ht="24.75" thickBot="1">
       <c r="A48" s="1"/>
       <c r="B48" s="11">
         <f>ROW(B48) - ROW($B$2)</f>
@@ -3772,7 +3819,7 @@
       </c>
       <c r="K48" s="7"/>
     </row>
-    <row r="49" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:11" ht="15.75" thickBot="1">
       <c r="A49" s="1"/>
       <c r="B49" s="11">
         <f t="shared" si="0"/>
@@ -3806,7 +3853,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="50" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:11" ht="24.75" thickBot="1">
       <c r="A50" s="1"/>
       <c r="B50" s="11">
         <f>ROW(B50) - ROW($B$2)</f>
@@ -3838,7 +3885,7 @@
       </c>
       <c r="K50" s="7"/>
     </row>
-    <row r="51" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:11" ht="24.75" thickBot="1">
       <c r="A51" s="1"/>
       <c r="B51" s="11">
         <f t="shared" si="0"/>
@@ -3870,7 +3917,7 @@
       </c>
       <c r="K51" s="9"/>
     </row>
-    <row r="52" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:11" ht="24.75" thickBot="1">
       <c r="A52" s="1"/>
       <c r="B52" s="11">
         <f>ROW(B52) - ROW($B$2)</f>
@@ -3902,7 +3949,7 @@
       </c>
       <c r="K52" s="7"/>
     </row>
-    <row r="53" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:11" ht="15.75" thickBot="1">
       <c r="A53" s="1"/>
       <c r="B53" s="11">
         <f t="shared" si="0"/>
@@ -3934,7 +3981,7 @@
       </c>
       <c r="K53" s="9"/>
     </row>
-    <row r="54" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:11" ht="24.75" thickBot="1">
       <c r="A54" s="1"/>
       <c r="B54" s="11">
         <f>ROW(B54) - ROW($B$2)</f>
@@ -3966,7 +4013,7 @@
       </c>
       <c r="K54" s="7"/>
     </row>
-    <row r="55" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:11" ht="36.75" thickBot="1">
       <c r="A55" s="1"/>
       <c r="B55" s="11">
         <f t="shared" si="0"/>
@@ -3998,7 +4045,7 @@
       </c>
       <c r="K55" s="9"/>
     </row>
-    <row r="56" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:11" ht="15.75" thickBot="1">
       <c r="A56" s="1"/>
       <c r="B56" s="11">
         <f>ROW(B56) - ROW($B$2)</f>
@@ -4030,7 +4077,7 @@
       </c>
       <c r="K56" s="7"/>
     </row>
-    <row r="57" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:11" ht="15.75" thickBot="1">
       <c r="A57" s="1"/>
       <c r="B57" s="11">
         <f t="shared" si="0"/>
@@ -4062,7 +4109,7 @@
       </c>
       <c r="K57" s="9"/>
     </row>
-    <row r="58" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:11" ht="15.75" thickBot="1">
       <c r="A58" s="1"/>
       <c r="B58" s="11">
         <f>ROW(B58) - ROW($B$2)</f>
@@ -4094,7 +4141,7 @@
       </c>
       <c r="K58" s="7"/>
     </row>
-    <row r="59" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:11" ht="15.75" thickBot="1">
       <c r="A59" s="1"/>
       <c r="B59" s="11">
         <f t="shared" si="0"/>
@@ -4126,7 +4173,7 @@
       </c>
       <c r="K59" s="9"/>
     </row>
-    <row r="60" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:11" ht="15.75" thickBot="1">
       <c r="A60" s="1"/>
       <c r="B60" s="11">
         <f>ROW(B60) - ROW($B$2)</f>
@@ -4158,7 +4205,7 @@
       </c>
       <c r="K60" s="7"/>
     </row>
-    <row r="61" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:11" ht="15.75" thickBot="1">
       <c r="A61" s="1"/>
       <c r="B61" s="11">
         <f t="shared" si="0"/>
@@ -4190,7 +4237,7 @@
       </c>
       <c r="K61" s="9"/>
     </row>
-    <row r="62" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:11" ht="15.75" thickBot="1">
       <c r="A62" s="1"/>
       <c r="B62" s="11">
         <f>ROW(B62) - ROW($B$2)</f>
@@ -4222,7 +4269,7 @@
       </c>
       <c r="K62" s="7"/>
     </row>
-    <row r="63" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:11" ht="15.75" thickBot="1">
       <c r="A63" s="1"/>
       <c r="B63" s="11">
         <f t="shared" si="0"/>
@@ -4254,7 +4301,7 @@
       </c>
       <c r="K63" s="9"/>
     </row>
-    <row r="64" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:11" ht="15.75" thickBot="1">
       <c r="A64" s="1"/>
       <c r="B64" s="11">
         <f>ROW(B64) - ROW($B$2)</f>
@@ -4286,7 +4333,7 @@
       </c>
       <c r="K64" s="7"/>
     </row>
-    <row r="65" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:11" ht="15.75" thickBot="1">
       <c r="A65" s="1"/>
       <c r="B65" s="11">
         <f t="shared" si="0"/>
@@ -4318,7 +4365,7 @@
       </c>
       <c r="K65" s="9"/>
     </row>
-    <row r="66" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:11" ht="15.75" thickBot="1">
       <c r="A66" s="1"/>
       <c r="B66" s="11">
         <f>ROW(B66) - ROW($B$2)</f>
@@ -4350,7 +4397,7 @@
       </c>
       <c r="K66" s="7"/>
     </row>
-    <row r="67" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:11" ht="15.75" thickBot="1">
       <c r="A67" s="1"/>
       <c r="B67" s="11">
         <f t="shared" si="0"/>
@@ -4382,7 +4429,7 @@
       </c>
       <c r="K67" s="9"/>
     </row>
-    <row r="68" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:11" ht="15.75" thickBot="1">
       <c r="A68" s="1"/>
       <c r="B68" s="11">
         <f>ROW(B68) - ROW($B$2)</f>
@@ -4414,7 +4461,7 @@
       </c>
       <c r="K68" s="7"/>
     </row>
-    <row r="69" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:11" ht="15.75" thickBot="1">
       <c r="A69" s="1"/>
       <c r="B69" s="11">
         <f t="shared" si="0"/>
@@ -4446,7 +4493,7 @@
       </c>
       <c r="K69" s="9"/>
     </row>
-    <row r="70" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:11" ht="15.75" thickBot="1">
       <c r="A70" s="1"/>
       <c r="B70" s="11">
         <f>ROW(B70) - ROW($B$2)</f>
@@ -4478,7 +4525,7 @@
       </c>
       <c r="K70" s="7"/>
     </row>
-    <row r="71" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:11" ht="36.75" thickBot="1">
       <c r="A71" s="1"/>
       <c r="B71" s="11">
         <f t="shared" si="0"/>
@@ -4510,7 +4557,7 @@
       </c>
       <c r="K71" s="9"/>
     </row>
-    <row r="72" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:11" ht="15.75" thickBot="1">
       <c r="A72" s="1"/>
       <c r="B72" s="11">
         <f>ROW(B72) - ROW($B$2)</f>
@@ -4542,7 +4589,7 @@
       </c>
       <c r="K72" s="7"/>
     </row>
-    <row r="73" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:11" ht="15.75" thickBot="1">
       <c r="A73" s="1"/>
       <c r="B73" s="11">
         <f t="shared" si="0"/>
@@ -4574,7 +4621,7 @@
       </c>
       <c r="K73" s="9"/>
     </row>
-    <row r="74" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:11" ht="15.75" thickBot="1">
       <c r="A74" s="1"/>
       <c r="B74" s="11">
         <f>ROW(B74) - ROW($B$2)</f>
@@ -4606,7 +4653,7 @@
       </c>
       <c r="K74" s="7"/>
     </row>
-    <row r="75" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:11" ht="24.75" thickBot="1">
       <c r="A75" s="1"/>
       <c r="B75" s="11">
         <f t="shared" si="0"/>
@@ -4638,7 +4685,7 @@
       </c>
       <c r="K75" s="9"/>
     </row>
-    <row r="76" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:11" ht="15.75" thickBot="1">
       <c r="A76" s="1"/>
       <c r="B76" s="11">
         <f>ROW(B76) - ROW($B$2)</f>
@@ -4670,7 +4717,7 @@
       </c>
       <c r="K76" s="7"/>
     </row>
-    <row r="77" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:11" ht="15.75" thickBot="1">
       <c r="A77" s="1"/>
       <c r="B77" s="11">
         <f t="shared" si="0"/>
@@ -4702,7 +4749,7 @@
       </c>
       <c r="K77" s="9"/>
     </row>
-    <row r="78" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:11" ht="15.75" thickBot="1">
       <c r="A78" s="1"/>
       <c r="B78" s="11">
         <f>ROW(B78) - ROW($B$2)</f>
@@ -4734,7 +4781,7 @@
       </c>
       <c r="K78" s="7"/>
     </row>
-    <row r="79" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:11" ht="15.75" thickBot="1">
       <c r="A79" s="1"/>
       <c r="B79" s="11">
         <f t="shared" si="0"/>
@@ -4766,7 +4813,7 @@
       </c>
       <c r="K79" s="9"/>
     </row>
-    <row r="80" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:11" ht="15.75" thickBot="1">
       <c r="A80" s="1"/>
       <c r="B80" s="11">
         <f>ROW(B80) - ROW($B$2)</f>
@@ -4798,7 +4845,7 @@
       </c>
       <c r="K80" s="7"/>
     </row>
-    <row r="81" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:11" ht="15.75" thickBot="1">
       <c r="A81" s="1"/>
       <c r="B81" s="11">
         <f t="shared" si="0"/>
@@ -4830,7 +4877,7 @@
       </c>
       <c r="K81" s="9"/>
     </row>
-    <row r="82" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:11" ht="15.75" thickBot="1">
       <c r="A82" s="1"/>
       <c r="B82" s="11">
         <f>ROW(B82) - ROW($B$2)</f>
@@ -4862,7 +4909,7 @@
       </c>
       <c r="K82" s="7"/>
     </row>
-    <row r="83" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:11" ht="15.75" thickBot="1">
       <c r="A83" s="1"/>
       <c r="B83" s="11">
         <f t="shared" si="0"/>
@@ -4894,7 +4941,7 @@
       </c>
       <c r="K83" s="9"/>
     </row>
-    <row r="84" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:11" ht="15.75" thickBot="1">
       <c r="A84" s="1"/>
       <c r="B84" s="11">
         <f>ROW(B84) - ROW($B$2)</f>
@@ -4926,7 +4973,7 @@
       </c>
       <c r="K84" s="7"/>
     </row>
-    <row r="85" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:11" ht="15.75" thickBot="1">
       <c r="A85" s="1"/>
       <c r="B85" s="11">
         <f t="shared" si="0"/>
@@ -4958,7 +5005,7 @@
       </c>
       <c r="K85" s="9"/>
     </row>
-    <row r="86" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:11" ht="15.75" thickBot="1">
       <c r="A86" s="1"/>
       <c r="B86" s="11">
         <f>ROW(B86) - ROW($B$2)</f>
@@ -4990,7 +5037,7 @@
       </c>
       <c r="K86" s="7"/>
     </row>
-    <row r="87" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:11" ht="15.75" thickBot="1">
       <c r="A87" s="1"/>
       <c r="B87" s="11">
         <f t="shared" si="0"/>
@@ -5022,7 +5069,7 @@
       </c>
       <c r="K87" s="9"/>
     </row>
-    <row r="88" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:11" ht="15.75" thickBot="1">
       <c r="A88" s="1"/>
       <c r="B88" s="11">
         <f>ROW(B88) - ROW($B$2)</f>
@@ -5054,7 +5101,7 @@
       </c>
       <c r="K88" s="7"/>
     </row>
-    <row r="89" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:11" ht="15.75" thickBot="1">
       <c r="A89" s="1"/>
       <c r="B89" s="11">
         <f t="shared" si="0"/>
@@ -5086,7 +5133,7 @@
       </c>
       <c r="K89" s="9"/>
     </row>
-    <row r="90" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:11" ht="15.75" thickBot="1">
       <c r="A90" s="1"/>
       <c r="B90" s="11">
         <f>ROW(B90) - ROW($B$2)</f>
@@ -5118,7 +5165,7 @@
       </c>
       <c r="K90" s="7"/>
     </row>
-    <row r="91" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:11" ht="15.75" thickBot="1">
       <c r="A91" s="1"/>
       <c r="B91" s="11">
         <f t="shared" si="0"/>
@@ -5150,7 +5197,7 @@
       </c>
       <c r="K91" s="9"/>
     </row>
-    <row r="92" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:11" ht="15.75" thickBot="1">
       <c r="A92" s="1"/>
       <c r="B92" s="11">
         <f>ROW(B92) - ROW($B$2)</f>
@@ -5182,7 +5229,7 @@
       </c>
       <c r="K92" s="7"/>
     </row>
-    <row r="93" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:11" ht="15.75" thickBot="1">
       <c r="A93" s="1"/>
       <c r="B93" s="11">
         <f t="shared" si="0"/>
@@ -5214,7 +5261,7 @@
       </c>
       <c r="K93" s="9"/>
     </row>
-    <row r="94" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:11" ht="15.75" thickBot="1">
       <c r="A94" s="1"/>
       <c r="B94" s="11">
         <f>ROW(B94) - ROW($B$2)</f>
@@ -5246,7 +5293,7 @@
       </c>
       <c r="K94" s="7"/>
     </row>
-    <row r="95" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:11" ht="15.75" thickBot="1">
       <c r="A95" s="1"/>
       <c r="B95" s="11">
         <f t="shared" si="0"/>
@@ -5278,7 +5325,7 @@
       </c>
       <c r="K95" s="9"/>
     </row>
-    <row r="96" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:11" ht="15.75" thickBot="1">
       <c r="A96" s="1"/>
       <c r="B96" s="11">
         <f>ROW(B96) - ROW($B$2)</f>
@@ -5310,7 +5357,7 @@
       </c>
       <c r="K96" s="7"/>
     </row>
-    <row r="97" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:11" ht="15.75" thickBot="1">
       <c r="A97" s="1"/>
       <c r="B97" s="11">
         <f t="shared" si="0"/>
@@ -5342,7 +5389,7 @@
       </c>
       <c r="K97" s="9"/>
     </row>
-    <row r="98" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:11" ht="15.75" thickBot="1">
       <c r="A98" s="1"/>
       <c r="B98" s="11">
         <f>ROW(B98) - ROW($B$2)</f>
@@ -5376,7 +5423,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="99" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:11" ht="36.75" thickBot="1">
       <c r="A99" s="1"/>
       <c r="B99" s="11">
         <f t="shared" si="0"/>
@@ -5408,7 +5455,7 @@
       </c>
       <c r="K99" s="9"/>
     </row>
-    <row r="100" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:11" ht="15.75" thickBot="1">
       <c r="A100" s="1"/>
       <c r="B100" s="11">
         <f>ROW(B100) - ROW($B$2)</f>
@@ -5440,7 +5487,7 @@
       </c>
       <c r="K100" s="7"/>
     </row>
-    <row r="101" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:11" ht="15.75" thickBot="1">
       <c r="A101" s="1"/>
       <c r="B101" s="11">
         <f t="shared" si="0"/>
@@ -5472,7 +5519,7 @@
       </c>
       <c r="K101" s="9"/>
     </row>
-    <row r="102" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:11" ht="15.75" thickBot="1">
       <c r="A102" s="1"/>
       <c r="B102" s="11">
         <f>ROW(B102) - ROW($B$2)</f>
@@ -5504,7 +5551,7 @@
       </c>
       <c r="K102" s="7"/>
     </row>
-    <row r="103" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:11" ht="15.75" thickBot="1">
       <c r="A103" s="1"/>
       <c r="B103" s="11">
         <f t="shared" si="0"/>
@@ -5538,7 +5585,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="104" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:11" ht="15.75" thickBot="1">
       <c r="A104" s="1"/>
       <c r="B104" s="11">
         <f>ROW(B104) - ROW($B$2)</f>
@@ -5570,7 +5617,7 @@
       </c>
       <c r="K104" s="7"/>
     </row>
-    <row r="105" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:11" ht="15.75" thickBot="1">
       <c r="A105" s="1"/>
       <c r="B105" s="11">
         <f t="shared" si="0"/>
@@ -5604,7 +5651,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="106" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:11" ht="15.75" thickBot="1">
       <c r="A106" s="1"/>
       <c r="B106" s="11">
         <f>ROW(B106) - ROW($B$2)</f>
@@ -5636,7 +5683,7 @@
       </c>
       <c r="K106" s="7"/>
     </row>
-    <row r="107" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:11" ht="15.75" thickBot="1">
       <c r="A107" s="1"/>
       <c r="B107" s="11">
         <f t="shared" si="0"/>
@@ -5668,7 +5715,7 @@
       </c>
       <c r="K107" s="9"/>
     </row>
-    <row r="108" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:11" ht="15.75" thickBot="1">
       <c r="A108" s="1"/>
       <c r="B108" s="11">
         <f>ROW(B108) - ROW($B$2)</f>
@@ -5702,7 +5749,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="109" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:11" ht="15.75" thickBot="1">
       <c r="A109" s="1"/>
       <c r="B109" s="11">
         <f t="shared" si="0"/>
@@ -5736,7 +5783,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="110" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:11" ht="15.75" thickBot="1">
       <c r="A110" s="1"/>
       <c r="B110" s="11">
         <f t="shared" si="0"/>
@@ -5768,7 +5815,7 @@
       </c>
       <c r="K110" s="9"/>
     </row>
-    <row r="111" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:11" ht="24.75" thickBot="1">
       <c r="A111" s="1"/>
       <c r="B111" s="11">
         <f>ROW(B111) - ROW($B$2)</f>
@@ -5800,7 +5847,7 @@
       </c>
       <c r="K111" s="7"/>
     </row>
-    <row r="112" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:11" ht="48.75" thickBot="1">
       <c r="A112" s="1"/>
       <c r="B112" s="11">
         <f t="shared" si="0"/>
@@ -5832,7 +5879,7 @@
       </c>
       <c r="K112" s="9"/>
     </row>
-    <row r="113" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:11" ht="36.75" thickBot="1">
       <c r="A113" s="1"/>
       <c r="B113" s="11">
         <f>ROW(B113) - ROW($B$2)</f>
@@ -5864,7 +5911,7 @@
       </c>
       <c r="K113" s="7"/>
     </row>
-    <row r="114" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:11" ht="24.75" thickBot="1">
       <c r="A114" s="1"/>
       <c r="B114" s="11">
         <f t="shared" si="0"/>
@@ -5896,7 +5943,7 @@
       </c>
       <c r="K114" s="9"/>
     </row>
-    <row r="115" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:11" ht="15.75" thickBot="1">
       <c r="A115" s="1"/>
       <c r="B115" s="11">
         <f>ROW(B115) - ROW($B$2)</f>
@@ -5928,7 +5975,7 @@
       </c>
       <c r="K115" s="7"/>
     </row>
-    <row r="116" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:11" ht="15.75" thickBot="1">
       <c r="A116" s="1"/>
       <c r="B116" s="11">
         <f t="shared" si="0"/>
@@ -5960,7 +6007,7 @@
       </c>
       <c r="K116" s="9"/>
     </row>
-    <row r="117" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:11" ht="24.75" thickBot="1">
       <c r="A117" s="1"/>
       <c r="B117" s="11">
         <f>ROW(B117) - ROW($B$2)</f>
@@ -5992,7 +6039,7 @@
       </c>
       <c r="K117" s="7"/>
     </row>
-    <row r="118" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:11" ht="15.75" thickBot="1">
       <c r="A118" s="1"/>
       <c r="B118" s="11">
         <f t="shared" si="0"/>
@@ -6024,7 +6071,7 @@
       </c>
       <c r="K118" s="9"/>
     </row>
-    <row r="119" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:11" ht="15.75" thickBot="1">
       <c r="A119" s="1"/>
       <c r="B119" s="11">
         <f>ROW(B119) - ROW($B$2)</f>
@@ -6056,7 +6103,7 @@
       </c>
       <c r="K119" s="7"/>
     </row>
-    <row r="120" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:11" ht="15.75" thickBot="1">
       <c r="A120" s="1"/>
       <c r="B120" s="11">
         <f t="shared" si="0"/>
@@ -6088,7 +6135,7 @@
       </c>
       <c r="K120" s="9"/>
     </row>
-    <row r="121" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:11" ht="15.75" thickBot="1">
       <c r="A121" s="1"/>
       <c r="B121" s="11">
         <f>ROW(B121) - ROW($B$2)</f>
@@ -6120,7 +6167,7 @@
       </c>
       <c r="K121" s="7"/>
     </row>
-    <row r="122" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:11" ht="15.75" thickBot="1">
       <c r="A122" s="1"/>
       <c r="B122" s="11">
         <f t="shared" si="0"/>
@@ -6152,7 +6199,7 @@
       </c>
       <c r="K122" s="9"/>
     </row>
-    <row r="123" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:11" ht="15.75" thickBot="1">
       <c r="A123" s="1"/>
       <c r="B123" s="11">
         <f>ROW(B123) - ROW($B$2)</f>
@@ -6184,7 +6231,7 @@
       </c>
       <c r="K123" s="7"/>
     </row>
-    <row r="124" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:11" ht="24.75" thickBot="1">
       <c r="A124" s="1"/>
       <c r="B124" s="11">
         <f t="shared" si="0"/>
@@ -6216,7 +6263,7 @@
       </c>
       <c r="K124" s="9"/>
     </row>
-    <row r="125" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:11" ht="24.75" thickBot="1">
       <c r="A125" s="1"/>
       <c r="B125" s="11">
         <f>ROW(B125) - ROW($B$2)</f>
@@ -6248,7 +6295,7 @@
       </c>
       <c r="K125" s="7"/>
     </row>
-    <row r="126" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:11" ht="15.75" thickBot="1">
       <c r="A126" s="1"/>
       <c r="B126" s="11">
         <f t="shared" si="0"/>
@@ -6280,7 +6327,7 @@
       </c>
       <c r="K126" s="9"/>
     </row>
-    <row r="127" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:11" ht="24.75" thickBot="1">
       <c r="A127" s="1"/>
       <c r="B127" s="11">
         <f>ROW(B127) - ROW($B$2)</f>
@@ -6312,7 +6359,7 @@
       </c>
       <c r="K127" s="7"/>
     </row>
-    <row r="128" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:11" ht="15.75" thickBot="1">
       <c r="A128" s="1"/>
       <c r="B128" s="11">
         <f t="shared" si="0"/>
@@ -6344,7 +6391,7 @@
       </c>
       <c r="K128" s="9"/>
     </row>
-    <row r="129" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:11" ht="36.75" thickBot="1">
       <c r="A129" s="1"/>
       <c r="B129" s="11">
         <f t="shared" si="0"/>
@@ -6376,7 +6423,7 @@
       </c>
       <c r="K129" s="9"/>
     </row>
-    <row r="130" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:11" ht="15.75" thickBot="1">
       <c r="A130" s="1"/>
       <c r="B130" s="11">
         <f>ROW(B130) - ROW($B$2)</f>
@@ -6408,7 +6455,7 @@
       </c>
       <c r="K130" s="7"/>
     </row>
-    <row r="131" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:11" ht="36.75" thickBot="1">
       <c r="A131" s="1"/>
       <c r="B131" s="11">
         <f t="shared" si="0"/>
@@ -6440,7 +6487,7 @@
       </c>
       <c r="K131" s="9"/>
     </row>
-    <row r="132" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:11" ht="24.75" thickBot="1">
       <c r="B132" s="11">
         <f>ROW(B132) - ROW($B$2)</f>
         <v>130</v>
@@ -6471,7 +6518,7 @@
       </c>
       <c r="K132" s="7"/>
     </row>
-    <row r="133" spans="1:11" ht="64.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:11" ht="64.5" thickBot="1">
       <c r="B133" s="11">
         <f>ROW(B133) - ROW($B$2)</f>
         <v>131</v>
@@ -6504,9 +6551,9 @@
         <v>549</v>
       </c>
     </row>
-    <row r="134" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:11" ht="36.75" thickBot="1">
       <c r="B134" s="11">
-        <f t="shared" ref="B134:B135" si="1">ROW(B134) - ROW($B$2)</f>
+        <f t="shared" ref="B134:B136" si="1">ROW(B134) - ROW($B$2)</f>
         <v>132</v>
       </c>
       <c r="C134" s="12" t="s">
@@ -6535,7 +6582,7 @@
       </c>
       <c r="K134" s="9"/>
     </row>
-    <row r="135" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:11" ht="24.75" thickBot="1">
       <c r="B135" s="11">
         <f t="shared" si="1"/>
         <v>133</v>
@@ -6565,12 +6612,48 @@
         <v>2</v>
       </c>
       <c r="K135" s="9"/>
+    </row>
+    <row r="136" spans="1:11" ht="36.75" thickBot="1">
+      <c r="B136" s="11">
+        <f t="shared" si="1"/>
+        <v>134</v>
+      </c>
+      <c r="C136" s="12" t="s">
+        <v>542</v>
+      </c>
+      <c r="D136" s="7" t="s">
+        <v>541</v>
+      </c>
+      <c r="E136" s="10" t="s">
+        <v>561</v>
+      </c>
+      <c r="F136" s="9" t="s">
+        <v>540</v>
+      </c>
+      <c r="G136" s="10" t="s">
+        <v>562</v>
+      </c>
+      <c r="H136" s="9" t="s">
+        <v>563</v>
+      </c>
+      <c r="I136" s="10" t="s">
+        <v>541</v>
+      </c>
+      <c r="J136" s="9">
+        <v>1</v>
+      </c>
+      <c r="K136" s="19" t="s">
+        <v>564</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="I1:K1"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="K136" r:id="rId1" location="nav-specification"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
#13 LCD Peripheral added.
</commit_message>
<xml_diff>
--- a/Design-Files/OFP_MCM_v1.5/BOM/Client-BOM-OFP_MCM_v1.5.xlsx
+++ b/Design-Files/OFP_MCM_v1.5/BOM/Client-BOM-OFP_MCM_v1.5.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="967" uniqueCount="566">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="975" uniqueCount="570">
   <si>
     <t>#</t>
   </si>
@@ -1717,6 +1717,18 @@
   </si>
   <si>
     <t>R85</t>
+  </si>
+  <si>
+    <t>5 inch TFT LCD Display 800*480 RGB Interface LCD Touch Screen Panel</t>
+  </si>
+  <si>
+    <t>RGB5001</t>
+  </si>
+  <si>
+    <t>QDTFT</t>
+  </si>
+  <si>
+    <t>Alibaba</t>
   </si>
 </sst>
 </file>
@@ -2281,7 +2293,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:U137"/>
+  <dimension ref="A1:U138"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="4" style="4" bestFit="1" customWidth="1"/>
@@ -7043,7 +7055,7 @@
       </c>
       <c r="K132" s="9"/>
       <c r="U132" t="b">
-        <f t="shared" ref="T132:U137" si="3">IF(P132=J132,TRUE,FALSE)</f>
+        <f t="shared" ref="U132:U138" si="3">IF(P132=J132,TRUE,FALSE)</f>
         <v>0</v>
       </c>
     </row>
@@ -7121,7 +7133,7 @@
     </row>
     <row r="135" spans="1:21" ht="36.75" thickBot="1">
       <c r="B135" s="11">
-        <f t="shared" ref="B135:B137" si="4">ROW(B135) - ROW($B$2)</f>
+        <f t="shared" ref="B135:B138" si="4">ROW(B135) - ROW($B$2)</f>
         <v>133</v>
       </c>
       <c r="C135" s="12" t="s">
@@ -7222,6 +7234,43 @@
         <v>561</v>
       </c>
       <c r="U137" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="138" spans="1:21" ht="24.75" thickBot="1">
+      <c r="B138" s="11">
+        <f t="shared" si="4"/>
+        <v>136</v>
+      </c>
+      <c r="C138" s="12" t="s">
+        <v>539</v>
+      </c>
+      <c r="D138" s="7" t="s">
+        <v>538</v>
+      </c>
+      <c r="E138" s="10" t="s">
+        <v>566</v>
+      </c>
+      <c r="F138" s="9" t="s">
+        <v>537</v>
+      </c>
+      <c r="G138" s="10" t="s">
+        <v>567</v>
+      </c>
+      <c r="H138" s="9" t="s">
+        <v>568</v>
+      </c>
+      <c r="I138" s="10" t="s">
+        <v>538</v>
+      </c>
+      <c r="J138" s="9">
+        <v>1</v>
+      </c>
+      <c r="K138" s="18" t="s">
+        <v>569</v>
+      </c>
+      <c r="U138" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -7232,8 +7281,9 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="K137" r:id="rId1" location="nav-specification"/>
+    <hyperlink ref="K138" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>